<commit_message>
removed ambig sets uncertainty prop. and added w2 errors at time steps
</commit_message>
<xml_diff>
--- a/examples/benchmark_results/gmm_discretization_results_test_2025-06-23_1_experiment1.xlsx
+++ b/examples/benchmark_results/gmm_discretization_results_test_2025-06-23_1_experiment1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elizealwash/PycharmProjects/discretize_distributions_new/examples/benchmark_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6463AA93-0C0C-A642-89A0-3948D91DB0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACE7966-0B15-354F-8051-C5B2337CBECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="15880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>run</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>nr_locs_old</t>
+  </si>
+  <si>
+    <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>STTDEV</t>
   </si>
 </sst>
 </file>
@@ -3356,6 +3362,9 @@
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C103" t="s">
+        <v>9</v>
+      </c>
       <c r="D103">
         <f>AVERAGE((D2:D101))</f>
         <v>0.39916792124509809</v>
@@ -3382,6 +3391,9 @@
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C104" t="s">
+        <v>10</v>
+      </c>
       <c r="D104">
         <f>STDEV(D2:D101)</f>
         <v>4.3339960920808523E-2</v>

</xml_diff>